<commit_message>
Update inventory, sales, and reports
</commit_message>
<xml_diff>
--- a/reports/sales_excel_round_trip.xlsx
+++ b/reports/sales_excel_round_trip.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1186,6 +1186,314 @@
         <v>18</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>S014</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>90</v>
+      </c>
+      <c r="F18" t="n">
+        <v>45</v>
+      </c>
+      <c r="G18" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>90</v>
+      </c>
+      <c r="J18" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="K18" t="n">
+        <v>45</v>
+      </c>
+      <c r="L18" t="n">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>S014</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>45</v>
+      </c>
+      <c r="F19" t="n">
+        <v>25</v>
+      </c>
+      <c r="G19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Stationery</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>45</v>
+      </c>
+      <c r="J19" t="n">
+        <v>42.75</v>
+      </c>
+      <c r="K19" t="n">
+        <v>25</v>
+      </c>
+      <c r="L19" t="n">
+        <v>17.75</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>S014</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>P007</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="n">
+        <v>135</v>
+      </c>
+      <c r="F20" t="n">
+        <v>90</v>
+      </c>
+      <c r="G20" t="n">
+        <v>5</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>405</v>
+      </c>
+      <c r="J20" t="n">
+        <v>384.75</v>
+      </c>
+      <c r="K20" t="n">
+        <v>270</v>
+      </c>
+      <c r="L20" t="n">
+        <v>114.75</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>S015</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>180</v>
+      </c>
+      <c r="F21" t="n">
+        <v>110</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>180</v>
+      </c>
+      <c r="J21" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="K21" t="n">
+        <v>110</v>
+      </c>
+      <c r="L21" t="n">
+        <v>66.40000000000001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>S015</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>45</v>
+      </c>
+      <c r="F22" t="n">
+        <v>25</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Stationery</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>45</v>
+      </c>
+      <c r="J22" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="K22" t="n">
+        <v>25</v>
+      </c>
+      <c r="L22" t="n">
+        <v>19.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>S015</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>220</v>
+      </c>
+      <c r="F23" t="n">
+        <v>140</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>220</v>
+      </c>
+      <c r="J23" t="n">
+        <v>215.6</v>
+      </c>
+      <c r="K23" t="n">
+        <v>140</v>
+      </c>
+      <c r="L23" t="n">
+        <v>75.59999999999999</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>S015</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>P009</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>35</v>
+      </c>
+      <c r="F24" t="n">
+        <v>15</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Gifts</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>105</v>
+      </c>
+      <c r="J24" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="K24" t="n">
+        <v>45</v>
+      </c>
+      <c r="L24" t="n">
+        <v>57.89999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>